<commit_message>
С-29 form: match the user's filled sample
New blank template built from the user's filled example with all real data
removed (Times New Roman, extra line under the object, data row 28). The export
asks for header requisites (organisation, approver, object, part, act number,
МОЛ) and remembers them in the browser; the act number comes from the АВР.
Rows show «1 шт. = … м³; по АВР — … шт.» under the name, economy/overrun as
a signed value, and accounting codes with volumes in «Прим.».

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DLuSJnJDazQvZpuhFH5Xvd
</commit_message>
<xml_diff>
--- a/assets/templates/s29-blank.xlsx
+++ b/assets/templates/s29-blank.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Филимонова\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EB08BE8-6B02-4693-99BC-298F07DCD44D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{724A6343-8D33-440A-A4C9-924BFA3BC9B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{ECB51198-8F26-4281-85AE-3DB1B3DC9F05}"/>
   </bookViews>
@@ -18,38 +18,38 @@
   <definedNames>
     <definedName name="docGro" localSheetId="0">'С-29'!$A$12</definedName>
     <definedName name="docMonthYear" localSheetId="0">'С-29'!$D$11</definedName>
-    <definedName name="docName" localSheetId="0">'С-29'!$A$16</definedName>
-    <definedName name="docObj" localSheetId="0">'С-29'!$A$14</definedName>
+    <definedName name="docName" localSheetId="0">'С-29'!$A$18</definedName>
+    <definedName name="docObj" localSheetId="0">'С-29'!$A$16</definedName>
     <definedName name="forContractor" localSheetId="0">'С-29'!$A$2</definedName>
     <definedName name="signAffirmFio" localSheetId="0">'С-29'!$H$5</definedName>
     <definedName name="signAffirmPic" localSheetId="0">'С-29'!$G$5</definedName>
     <definedName name="signAffirmPos" localSheetId="0">'С-29'!$E$5</definedName>
     <definedName name="signDateAffirm" localSheetId="0">'С-29'!$F$8</definedName>
-    <definedName name="signDateCompose" comment="подпись Дата составления" localSheetId="0">'С-29'!$D$33</definedName>
-    <definedName name="signDatePassToBuh" comment="подпись Дата передачи в бухгалтерию" localSheetId="0">'С-29'!$D$35</definedName>
-    <definedName name="signEngineerPTOfio" localSheetId="0">'С-29'!$F$30</definedName>
-    <definedName name="signEngineerPTOpic" comment="подпись Инженер ПТО" localSheetId="0">'С-29'!$D$30</definedName>
-    <definedName name="signEngineerPTOpos" localSheetId="0">'С-29'!$A$30</definedName>
-    <definedName name="signMOLfio" localSheetId="0">'С-29'!$F$27</definedName>
-    <definedName name="signMOLFioHeader" localSheetId="0">'С-29'!$G$18:$I$18</definedName>
-    <definedName name="signMOLpic" comment="подпись Материально ответственное лицо" localSheetId="0">'С-29'!$D$27</definedName>
-    <definedName name="signMOLPosHeader" comment="в шапке Материально ответственное лицо" localSheetId="0">'С-29'!$D$18:$F$18</definedName>
-    <definedName name="smwCount" localSheetId="0">'С-29'!$F$21</definedName>
-    <definedName name="smwEd" localSheetId="0">'С-29'!$D$21</definedName>
-    <definedName name="smwLab" localSheetId="0">'С-29'!$B$21</definedName>
-    <definedName name="smwName" localSheetId="0">'С-29'!$C$21</definedName>
-    <definedName name="smwNpp" localSheetId="0">'С-29'!$A$21</definedName>
-    <definedName name="smwrPrim" localSheetId="0">'С-29'!$H$21</definedName>
-    <definedName name="smwrTotalCount" localSheetId="0">'С-29'!$G$21</definedName>
-    <definedName name="wrsDivCount" localSheetId="0">'С-29'!$G$26</definedName>
-    <definedName name="wrsEd" localSheetId="0">'С-29'!$D$26</definedName>
-    <definedName name="wrsFCount" localSheetId="0">'С-29'!$F$26</definedName>
-    <definedName name="wrsLab" localSheetId="0">'С-29'!$B$26</definedName>
-    <definedName name="wrsName" localSheetId="0">'С-29'!$C$26</definedName>
-    <definedName name="wrsNpp" localSheetId="0">'С-29'!$A$26</definedName>
-    <definedName name="wrsPrim" localSheetId="0">'С-29'!$I$26</definedName>
-    <definedName name="wrsSCount" localSheetId="0">'С-29'!$E$26</definedName>
-    <definedName name="wrsWriteOff" localSheetId="0">'С-29'!$H$26</definedName>
+    <definedName name="signDateCompose" comment="подпись Дата составления" localSheetId="0">'С-29'!$D$36</definedName>
+    <definedName name="signDatePassToBuh" comment="подпись Дата передачи в бухгалтерию" localSheetId="0">'С-29'!$D$38</definedName>
+    <definedName name="signEngineerPTOfio" localSheetId="0">'С-29'!$F$33</definedName>
+    <definedName name="signEngineerPTOpic" comment="подпись Инженер ПТО" localSheetId="0">'С-29'!$D$33</definedName>
+    <definedName name="signEngineerPTOpos" localSheetId="0">'С-29'!$A$33</definedName>
+    <definedName name="signMOLfio" localSheetId="0">'С-29'!$F$30</definedName>
+    <definedName name="signMOLFioHeader" localSheetId="0">'С-29'!$G$20:$I$20</definedName>
+    <definedName name="signMOLpic" comment="подпись Материально ответственное лицо" localSheetId="0">'С-29'!$D$30</definedName>
+    <definedName name="signMOLPosHeader" comment="в шапке Материально ответственное лицо" localSheetId="0">'С-29'!$D$20:$F$20</definedName>
+    <definedName name="smwCount" localSheetId="0">'С-29'!$F$23</definedName>
+    <definedName name="smwEd" localSheetId="0">'С-29'!$D$23</definedName>
+    <definedName name="smwLab" localSheetId="0">'С-29'!$B$23</definedName>
+    <definedName name="smwName" localSheetId="0">'С-29'!$C$23</definedName>
+    <definedName name="smwNpp" localSheetId="0">'С-29'!$A$23</definedName>
+    <definedName name="smwrPrim" localSheetId="0">'С-29'!$H$23</definedName>
+    <definedName name="smwrTotalCount" localSheetId="0">'С-29'!$G$23</definedName>
+    <definedName name="wrsDivCount" localSheetId="0">'С-29'!$G$28</definedName>
+    <definedName name="wrsEd" localSheetId="0">'С-29'!$D$28</definedName>
+    <definedName name="wrsFCount" localSheetId="0">'С-29'!$F$28</definedName>
+    <definedName name="wrsLab" localSheetId="0">'С-29'!$B$28</definedName>
+    <definedName name="wrsName" localSheetId="0">'С-29'!$C$28</definedName>
+    <definedName name="wrsNpp" localSheetId="0">'С-29'!$A$28</definedName>
+    <definedName name="wrsPrim" localSheetId="0">'С-29'!$I$28</definedName>
+    <definedName name="wrsSCount" localSheetId="0">'С-29'!$E$28</definedName>
+    <definedName name="wrsWriteOff" localSheetId="0">'С-29'!$H$28</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -75,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="47">
   <si>
     <t>Форма С-29</t>
   </si>
@@ -104,9 +104,6 @@
     <t>о расходе строительных материалов в сопоставлении с нормами</t>
   </si>
   <si>
-    <t>Объект строительства:</t>
-  </si>
-  <si>
     <t>(наименование объекта строительства)</t>
   </si>
   <si>
@@ -116,9 +113,6 @@
     <t>(наименование части объекта строительства)</t>
   </si>
   <si>
-    <t>Номер и наименование акта:</t>
-  </si>
-  <si>
     <t>Материально ответственное лицо:</t>
   </si>
   <si>
@@ -177,16 +171,58 @@
   </si>
   <si>
     <t>Дата передачи в бухгалтерию</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0.000"/>
-  </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial Cyr"/>
@@ -194,26 +230,40 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
       <charset val="204"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
       <charset val="204"/>
     </font>
     <font>
       <sz val="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
       <charset val="204"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
       <charset val="204"/>
     </font>
   </fonts>
@@ -357,7 +407,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -369,17 +419,35 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -398,74 +466,59 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -804,8 +857,8 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:I38"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.88671875" style="3" customWidth="1"/>
     <col min="2" max="2" width="12.88671875" style="3" customWidth="1"/>
@@ -813,11 +866,11 @@
     <col min="4" max="5" width="9.6640625" style="3" customWidth="1"/>
     <col min="6" max="7" width="12.6640625" style="3" customWidth="1"/>
     <col min="8" max="8" width="9.6640625" style="3" customWidth="1"/>
-    <col min="9" max="9" width="10.6640625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="20.5546875" style="3" customWidth="1"/>
     <col min="10" max="16384" width="9.109375" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="2"/>
@@ -827,20 +880,20 @@
       </c>
       <c r="H1" s="1"/>
     </row>
-    <row r="2" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="4"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="32" t="s">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="32"/>
-      <c r="C3" s="32"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
       <c r="E3" s="1" t="s">
         <v>2</v>
       </c>
@@ -848,7 +901,7 @@
       <c r="H3" s="6"/>
       <c r="I3" s="6"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="2"/>
@@ -857,33 +910,33 @@
       <c r="H4" s="6"/>
       <c r="I4" s="6"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="2"/>
-      <c r="E5" s="33"/>
-      <c r="F5" s="34"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="35"/>
-      <c r="I5" s="33"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E5" s="7"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="7"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="2"/>
-      <c r="E6" s="20" t="s">
+      <c r="E6" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="F6" s="20"/>
-      <c r="G6" s="8" t="s">
+      <c r="F6" s="11"/>
+      <c r="G6" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="H6" s="36" t="s">
+      <c r="H6" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="I6" s="36"/>
-    </row>
-    <row r="7" spans="1:9" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="I6" s="13"/>
+    </row>
+    <row r="7" spans="1:9" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="2"/>
@@ -892,7 +945,7 @@
       <c r="H7" s="6"/>
       <c r="I7" s="6"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="2"/>
@@ -905,329 +958,366 @@
       <c r="H8" s="6"/>
       <c r="I8" s="6"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="30" t="s">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="30"/>
-      <c r="C9" s="30"/>
-      <c r="D9" s="30"/>
-      <c r="E9" s="30"/>
-      <c r="F9" s="30"/>
-      <c r="G9" s="30"/>
-      <c r="H9" s="30"/>
-      <c r="I9" s="30"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="30" t="s">
+      <c r="B9" s="14"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="14"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="30"/>
-      <c r="C10" s="30"/>
-      <c r="D10" s="30"/>
-      <c r="E10" s="30"/>
-      <c r="F10" s="30"/>
-      <c r="G10" s="30"/>
-      <c r="H10" s="30"/>
-      <c r="I10" s="30"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
+      <c r="I10" s="14"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="10"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="16"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="11" t="s">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Объект строительства:</t>
+        </is>
+      </c>
+      <c r="B12" s="17"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="19"/>
+      <c r="B13" s="19"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="11"/>
-      <c r="I12" s="11"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="13"/>
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="14" t="s">
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="19"/>
+      <c r="I13" s="19"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="17"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="19"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="39"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="19"/>
+      <c r="H15" s="19"/>
+      <c r="I15" s="19"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
-      <c r="H13" s="13"/>
-      <c r="I13" s="13"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="11" t="s">
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="17"/>
+      <c r="I16" s="17"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="19"/>
+      <c r="B17" s="19"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="11"/>
-      <c r="I14" s="11"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" s="13"/>
-      <c r="B15" s="13"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="14" t="s">
+      <c r="E17" s="19"/>
+      <c r="F17" s="19"/>
+      <c r="G17" s="19"/>
+      <c r="H17" s="19"/>
+      <c r="I17" s="19"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Номер и наименование акта:</t>
+        </is>
+      </c>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="17"/>
+      <c r="I18" s="17"/>
+    </row>
+    <row r="19" spans="1:9" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D19" s="21"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="13"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="11"/>
-    </row>
-    <row r="17" spans="1:9" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D17" s="15"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A18" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D18" s="26"/>
-      <c r="E18" s="26"/>
-      <c r="F18" s="31"/>
-      <c r="G18" s="26"/>
-      <c r="H18" s="26"/>
-      <c r="I18" s="26"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="20" t="s">
-        <v>15</v>
-      </c>
-      <c r="H19" s="20"/>
-      <c r="I19" s="20"/>
-    </row>
-    <row r="20" spans="1:9" ht="9.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D20" s="22"/>
+      <c r="E20" s="22"/>
+      <c r="F20" s="23"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="22"/>
+      <c r="I20" s="22"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="I22" s="16" t="s">
+      <c r="C21" s="16"/>
+      <c r="D21" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="H21" s="11"/>
+      <c r="I21" s="11"/>
+    </row>
+    <row r="22" spans="1:9" ht="9.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="12"/>
+      <c r="H22" s="12"/>
+      <c r="I22" s="12"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I24" s="24" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="B25" s="26" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="D25" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="E25" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="F25" s="28"/>
+      <c r="G25" s="25" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="B23" s="27" t="s">
+      <c r="H25" s="25" t="s">
+        <v>22</v>
+      </c>
+      <c r="I25" s="25" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="29"/>
+      <c r="B26" s="26"/>
+      <c r="C26" s="29"/>
+      <c r="D26" s="29"/>
+      <c r="E26" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="F26" s="30" t="s">
+        <v>25</v>
+      </c>
+      <c r="G26" s="29"/>
+      <c r="H26" s="29"/>
+      <c r="I26" s="29"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="31">
+        <v>1</v>
+      </c>
+      <c r="B27" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="C23" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="D23" s="21" t="s">
-        <v>17</v>
-      </c>
-      <c r="E23" s="28" t="s">
-        <v>22</v>
-      </c>
-      <c r="F23" s="29"/>
-      <c r="G23" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="H23" s="21" t="s">
-        <v>24</v>
-      </c>
-      <c r="I23" s="21" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="22"/>
-      <c r="B24" s="27"/>
-      <c r="C24" s="22"/>
-      <c r="D24" s="22"/>
-      <c r="E24" s="17" t="s">
+      <c r="C27" s="31">
+        <v>3</v>
+      </c>
+      <c r="D27" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="F24" s="17" t="s">
+      <c r="E27" s="31">
+        <v>5</v>
+      </c>
+      <c r="F27" s="31">
+        <v>6</v>
+      </c>
+      <c r="G27" s="31">
+        <v>7</v>
+      </c>
+      <c r="H27" s="31">
+        <v>8</v>
+      </c>
+      <c r="I27" s="31">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="31"/>
+      <c r="B28" s="31"/>
+      <c r="C28" s="36"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="31"/>
+      <c r="F28" s="31"/>
+      <c r="G28" s="31"/>
+      <c r="H28" s="31"/>
+      <c r="I28" s="31"/>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" s="1"/>
+      <c r="B29" s="1"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="1"/>
+      <c r="I29" s="2"/>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="G24" s="22"/>
-      <c r="H24" s="22"/>
-      <c r="I24" s="22"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" s="18">
-        <v>1</v>
-      </c>
-      <c r="B25" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="C25" s="18">
-        <v>3</v>
-      </c>
-      <c r="D25" s="18" t="s">
+      <c r="D30" s="32"/>
+      <c r="E30" s="33"/>
+      <c r="F30" s="34"/>
+      <c r="G30" s="22"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D31" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="E31" s="11"/>
+      <c r="F31" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="G31" s="11"/>
+    </row>
+    <row r="32" spans="1:7" ht="9.9" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="E25" s="18">
-        <v>5</v>
-      </c>
-      <c r="F25" s="18">
-        <v>6</v>
-      </c>
-      <c r="G25" s="18">
-        <v>7</v>
-      </c>
-      <c r="H25" s="18">
-        <v>8</v>
-      </c>
-      <c r="I25" s="18">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A26" s="18"/>
-      <c r="B26" s="18"/>
-      <c r="C26" s="37"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="38"/>
-      <c r="F26" s="38"/>
-      <c r="G26" s="38"/>
-      <c r="H26" s="38"/>
-      <c r="I26" s="37"/>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" s="3" t="s">
+      <c r="D33" s="32"/>
+      <c r="E33" s="33"/>
+      <c r="F33" s="34"/>
+      <c r="G33" s="22"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D34" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="E34" s="11"/>
+      <c r="F34" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="G34" s="11"/>
+    </row>
+    <row r="35" spans="1:7" ht="9.9" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D27" s="23"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="25"/>
-      <c r="G27" s="26"/>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D28" s="20" t="s">
-        <v>4</v>
-      </c>
-      <c r="E28" s="20"/>
-      <c r="F28" s="20" t="s">
-        <v>15</v>
-      </c>
-      <c r="G28" s="20"/>
-    </row>
-    <row r="29" spans="1:9" ht="9.9" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" s="19" t="s">
+      <c r="D36" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D30" s="23"/>
-      <c r="E30" s="24"/>
-      <c r="F30" s="25"/>
-      <c r="G30" s="26"/>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D31" s="20" t="s">
-        <v>4</v>
-      </c>
-      <c r="E31" s="20"/>
-      <c r="F31" s="20" t="s">
-        <v>15</v>
-      </c>
-      <c r="G31" s="20"/>
-    </row>
-    <row r="32" spans="1:9" ht="9.9" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" s="3" t="s">
+    </row>
+    <row r="37" spans="1:7" ht="9.9" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D33" s="3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="9.9" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D35" s="3" t="s">
-        <v>32</v>
+      <c r="D38" s="3" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="H25:H26"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="I25:I26"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="A10:I10"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="G21:I21"/>
     <mergeCell ref="A9:I9"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="H5:I5"/>
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="H6:I6"/>
-    <mergeCell ref="A10:I10"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="G18:I18"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="C23:C24"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="G23:G24"/>
-    <mergeCell ref="H23:H24"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="I23:I24"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="F30:G30"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.59055118110236227" right="0.39370078740157483" top="0.39370078740157483" bottom="0.39370078740157483" header="0.19685039370078741" footer="0.19685039370078741"/>
-  <pageSetup paperSize="9" scale="80" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="74" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>